<commit_message>
Test Automation Framework - git CI/CD
</commit_message>
<xml_diff>
--- a/config/Master_Test_Template.xlsx
+++ b/config/Master_Test_Template.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="27928"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="28025"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gomat\PycharmProjects\test_automation_project\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CCD96A00-586C-4D15-9C52-26E0BA5F7B76}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C7C2C05-368E-4BD6-8128-E53D1B8E689D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -18,14 +18,14 @@
     <sheet name="data_quality_checks" sheetId="2" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">data_validation!$A$1:$W$29</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">data_validation!$A$1:$W$42</definedName>
   </definedNames>
   <calcPr calcId="144525"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="752" uniqueCount="101">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1037" uniqueCount="117">
   <si>
     <t>csv</t>
   </si>
@@ -327,19 +327,88 @@
     <t>N</t>
   </si>
   <si>
-    <t>Contact_info_26092024.csv</t>
+    <t>NY</t>
+  </si>
+  <si>
+    <t>date_check</t>
+  </si>
+  <si>
+    <t>YT01</t>
+  </si>
+  <si>
+    <t>adls</t>
+  </si>
+  <si>
+    <t>Contact_info_26102024.csv</t>
+  </si>
+  <si>
+    <t>FMT1</t>
+  </si>
+  <si>
+    <t>FMT2</t>
+  </si>
+  <si>
+    <t>FMT3</t>
+  </si>
+  <si>
+    <t>FMT4</t>
+  </si>
+  <si>
+    <t>FMT5</t>
+  </si>
+  <si>
+    <t>FMT6</t>
+  </si>
+  <si>
+    <t>FMT7</t>
+  </si>
+  <si>
+    <t>FMT8</t>
+  </si>
+  <si>
+    <t>FMT9</t>
+  </si>
+  <si>
+    <t>FMT10</t>
+  </si>
+  <si>
+    <t>FMT11</t>
+  </si>
+  <si>
+    <t>FMT12</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="31">
+  <fonts count="34">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -570,51 +639,69 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="41">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="23" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="49" fontId="20" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="18" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="0" applyFont="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="0" applyFont="1">
-      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -622,17 +709,11 @@
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="0" applyFont="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="49" fontId="15" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -642,9 +723,6 @@
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -656,7 +734,7 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -665,10 +743,14 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+      <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -676,12 +758,8 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -958,7 +1036,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:W37"/>
+  <dimension ref="A1:W50"/>
   <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="11.21875" style="2" bestFit="1" customWidth="1"/>
@@ -1059,14 +1137,14 @@
       </c>
     </row>
     <row r="2" spans="1:23">
-      <c r="A2" s="18" t="s">
-        <v>30</v>
+      <c r="A2" s="40" t="s">
+        <v>105</v>
       </c>
       <c r="B2" s="37" t="s">
         <v>25</v>
       </c>
       <c r="C2" s="24" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="D2" s="3" t="s">
         <v>0</v>
@@ -1084,16 +1162,16 @@
         <v>50</v>
       </c>
       <c r="I2" s="24" t="s">
-        <v>62</v>
+        <v>104</v>
       </c>
       <c r="J2" s="3" t="s">
-        <v>63</v>
+        <v>0</v>
       </c>
       <c r="K2" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="L2" s="24" t="s">
-        <v>64</v>
+      <c r="L2" s="3" t="s">
+        <v>17</v>
       </c>
       <c r="M2" s="3" t="s">
         <v>17</v>
@@ -1130,14 +1208,14 @@
       </c>
     </row>
     <row r="3" spans="1:23">
-      <c r="A3" s="18" t="s">
-        <v>40</v>
+      <c r="A3" s="40" t="s">
+        <v>106</v>
       </c>
       <c r="B3" s="37" t="s">
         <v>26</v>
       </c>
       <c r="C3" s="24" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="D3" s="3" t="s">
         <v>0</v>
@@ -1155,16 +1233,16 @@
         <v>50</v>
       </c>
       <c r="I3" s="24" t="s">
-        <v>62</v>
+        <v>104</v>
       </c>
       <c r="J3" s="3" t="s">
-        <v>63</v>
+        <v>0</v>
       </c>
       <c r="K3" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="L3" s="24" t="s">
-        <v>64</v>
+      <c r="L3" s="3" t="s">
+        <v>17</v>
       </c>
       <c r="M3" s="3" t="s">
         <v>17</v>
@@ -1201,14 +1279,14 @@
       </c>
     </row>
     <row r="4" spans="1:23">
-      <c r="A4" s="18" t="s">
-        <v>41</v>
+      <c r="A4" s="40" t="s">
+        <v>107</v>
       </c>
       <c r="B4" s="37" t="s">
         <v>27</v>
       </c>
       <c r="C4" s="24" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="D4" s="3" t="s">
         <v>0</v>
@@ -1226,16 +1304,16 @@
         <v>50</v>
       </c>
       <c r="I4" s="24" t="s">
-        <v>62</v>
+        <v>104</v>
       </c>
       <c r="J4" s="3" t="s">
-        <v>63</v>
+        <v>0</v>
       </c>
       <c r="K4" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="L4" s="24" t="s">
-        <v>64</v>
+      <c r="L4" s="3" t="s">
+        <v>17</v>
       </c>
       <c r="M4" s="3" t="s">
         <v>17</v>
@@ -1272,14 +1350,14 @@
       </c>
     </row>
     <row r="5" spans="1:23">
-      <c r="A5" s="18" t="s">
-        <v>42</v>
+      <c r="A5" s="40" t="s">
+        <v>108</v>
       </c>
       <c r="B5" s="37" t="s">
         <v>28</v>
       </c>
       <c r="C5" s="24" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="D5" s="3" t="s">
         <v>0</v>
@@ -1297,16 +1375,16 @@
         <v>50</v>
       </c>
       <c r="I5" s="24" t="s">
-        <v>62</v>
+        <v>104</v>
       </c>
       <c r="J5" s="3" t="s">
-        <v>63</v>
+        <v>0</v>
       </c>
       <c r="K5" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="L5" s="24" t="s">
-        <v>64</v>
+      <c r="L5" s="3" t="s">
+        <v>17</v>
       </c>
       <c r="M5" s="3" t="s">
         <v>17</v>
@@ -1343,14 +1421,14 @@
       </c>
     </row>
     <row r="6" spans="1:23">
-      <c r="A6" s="18" t="s">
-        <v>43</v>
+      <c r="A6" s="40" t="s">
+        <v>109</v>
       </c>
       <c r="B6" s="4" t="s">
         <v>29</v>
       </c>
       <c r="C6" s="24" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="D6" s="3" t="s">
         <v>0</v>
@@ -1368,16 +1446,16 @@
         <v>50</v>
       </c>
       <c r="I6" s="24" t="s">
-        <v>62</v>
+        <v>104</v>
       </c>
       <c r="J6" s="3" t="s">
-        <v>63</v>
+        <v>0</v>
       </c>
       <c r="K6" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="L6" s="24" t="s">
-        <v>64</v>
+      <c r="L6" s="3" t="s">
+        <v>17</v>
       </c>
       <c r="M6" s="3" t="s">
         <v>17</v>
@@ -1414,14 +1492,14 @@
       </c>
     </row>
     <row r="7" spans="1:23">
-      <c r="A7" s="18" t="s">
-        <v>44</v>
+      <c r="A7" s="40" t="s">
+        <v>110</v>
       </c>
       <c r="B7" s="4" t="s">
         <v>51</v>
       </c>
       <c r="C7" s="24" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="D7" s="3" t="s">
         <v>0</v>
@@ -1439,16 +1517,16 @@
         <v>50</v>
       </c>
       <c r="I7" s="24" t="s">
-        <v>62</v>
+        <v>104</v>
       </c>
       <c r="J7" s="3" t="s">
-        <v>63</v>
+        <v>0</v>
       </c>
       <c r="K7" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="L7" s="24" t="s">
-        <v>64</v>
+      <c r="L7" s="3" t="s">
+        <v>17</v>
       </c>
       <c r="M7" s="3" t="s">
         <v>17</v>
@@ -1485,14 +1563,14 @@
       </c>
     </row>
     <row r="8" spans="1:23">
-      <c r="A8" s="18" t="s">
-        <v>49</v>
+      <c r="A8" s="40" t="s">
+        <v>111</v>
       </c>
       <c r="B8" s="4" t="s">
         <v>52</v>
       </c>
       <c r="C8" s="24" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="D8" s="3" t="s">
         <v>0</v>
@@ -1510,16 +1588,16 @@
         <v>50</v>
       </c>
       <c r="I8" s="24" t="s">
-        <v>62</v>
+        <v>104</v>
       </c>
       <c r="J8" s="3" t="s">
-        <v>63</v>
+        <v>0</v>
       </c>
       <c r="K8" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="L8" s="24" t="s">
-        <v>64</v>
+      <c r="L8" s="3" t="s">
+        <v>17</v>
       </c>
       <c r="M8" s="3" t="s">
         <v>17</v>
@@ -1556,14 +1634,14 @@
       </c>
     </row>
     <row r="9" spans="1:23">
-      <c r="A9" s="32" t="s">
-        <v>54</v>
+      <c r="A9" s="40" t="s">
+        <v>112</v>
       </c>
       <c r="B9" s="37" t="s">
         <v>23</v>
       </c>
       <c r="C9" s="24" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="D9" s="3" t="s">
         <v>0</v>
@@ -1581,16 +1659,16 @@
         <v>50</v>
       </c>
       <c r="I9" s="24" t="s">
-        <v>62</v>
+        <v>104</v>
       </c>
       <c r="J9" s="3" t="s">
-        <v>63</v>
+        <v>0</v>
       </c>
       <c r="K9" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="L9" s="24" t="s">
-        <v>64</v>
+      <c r="L9" s="3" t="s">
+        <v>17</v>
       </c>
       <c r="M9" s="3" t="s">
         <v>17</v>
@@ -1627,14 +1705,14 @@
       </c>
     </row>
     <row r="10" spans="1:23">
-      <c r="A10" s="32" t="s">
-        <v>58</v>
+      <c r="A10" s="40" t="s">
+        <v>113</v>
       </c>
       <c r="B10" s="4" t="s">
         <v>55</v>
       </c>
       <c r="C10" s="24" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="D10" s="3" t="s">
         <v>0</v>
@@ -1652,16 +1730,16 @@
         <v>50</v>
       </c>
       <c r="I10" s="24" t="s">
-        <v>62</v>
+        <v>104</v>
       </c>
       <c r="J10" s="3" t="s">
-        <v>63</v>
+        <v>0</v>
       </c>
       <c r="K10" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="L10" s="24" t="s">
-        <v>64</v>
+      <c r="L10" s="3" t="s">
+        <v>17</v>
       </c>
       <c r="M10" s="3" t="s">
         <v>17</v>
@@ -1685,7 +1763,7 @@
         <v>2</v>
       </c>
       <c r="T10" s="3" t="s">
-        <v>17</v>
+        <v>84</v>
       </c>
       <c r="U10" s="3" t="s">
         <v>17</v>
@@ -1698,14 +1776,14 @@
       </c>
     </row>
     <row r="11" spans="1:23">
-      <c r="A11" s="32" t="s">
-        <v>59</v>
+      <c r="A11" s="40" t="s">
+        <v>114</v>
       </c>
       <c r="B11" s="4" t="s">
         <v>56</v>
       </c>
       <c r="C11" s="24" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="D11" s="3" t="s">
         <v>0</v>
@@ -1723,16 +1801,16 @@
         <v>50</v>
       </c>
       <c r="I11" s="24" t="s">
-        <v>62</v>
+        <v>104</v>
       </c>
       <c r="J11" s="3" t="s">
-        <v>63</v>
+        <v>0</v>
       </c>
       <c r="K11" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="L11" s="24" t="s">
-        <v>64</v>
+      <c r="L11" s="3" t="s">
+        <v>17</v>
       </c>
       <c r="M11" s="3" t="s">
         <v>17</v>
@@ -1756,27 +1834,27 @@
         <v>2</v>
       </c>
       <c r="T11" s="3" t="s">
-        <v>17</v>
+        <v>85</v>
       </c>
       <c r="U11" s="3" t="s">
         <v>17</v>
       </c>
       <c r="V11" s="2">
-        <v>0</v>
+        <v>19500000</v>
       </c>
       <c r="W11" s="2">
-        <v>0</v>
+        <v>20240930</v>
       </c>
     </row>
     <row r="12" spans="1:23">
-      <c r="A12" s="32" t="s">
-        <v>60</v>
+      <c r="A12" s="40" t="s">
+        <v>115</v>
       </c>
       <c r="B12" s="4" t="s">
         <v>57</v>
       </c>
       <c r="C12" s="24" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="D12" s="3" t="s">
         <v>0</v>
@@ -1794,16 +1872,16 @@
         <v>50</v>
       </c>
       <c r="I12" s="24" t="s">
-        <v>62</v>
+        <v>104</v>
       </c>
       <c r="J12" s="3" t="s">
-        <v>63</v>
+        <v>0</v>
       </c>
       <c r="K12" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="L12" s="24" t="s">
-        <v>64</v>
+      <c r="L12" s="3" t="s">
+        <v>17</v>
       </c>
       <c r="M12" s="3" t="s">
         <v>17</v>
@@ -1826,11 +1904,11 @@
       <c r="S12" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="T12" s="2" t="s">
-        <v>17</v>
+      <c r="T12" s="3" t="s">
+        <v>86</v>
       </c>
       <c r="U12" s="2" t="s">
-        <v>17</v>
+        <v>100</v>
       </c>
       <c r="V12" s="2">
         <v>0</v>
@@ -1840,41 +1918,41 @@
       </c>
     </row>
     <row r="13" spans="1:23">
-      <c r="A13" s="34" t="s">
-        <v>67</v>
-      </c>
-      <c r="B13" s="4" t="s">
-        <v>25</v>
+      <c r="A13" s="40" t="s">
+        <v>116</v>
+      </c>
+      <c r="B13" s="17" t="s">
+        <v>101</v>
       </c>
       <c r="C13" s="24" t="s">
-        <v>62</v>
+        <v>104</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>63</v>
+        <v>0</v>
       </c>
       <c r="E13" s="3" t="s">
         <v>17</v>
       </c>
       <c r="F13" s="3" t="s">
-        <v>64</v>
-      </c>
-      <c r="G13" s="34" t="s">
-        <v>78</v>
+        <v>17</v>
+      </c>
+      <c r="G13" s="3" t="s">
+        <v>17</v>
       </c>
       <c r="H13" s="3" t="s">
-        <v>17</v>
+        <v>50</v>
       </c>
       <c r="I13" s="24" t="s">
-        <v>66</v>
+        <v>104</v>
       </c>
       <c r="J13" s="3" t="s">
-        <v>63</v>
+        <v>0</v>
       </c>
       <c r="K13" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="L13" s="24" t="s">
-        <v>64</v>
+      <c r="L13" s="3" t="s">
+        <v>17</v>
       </c>
       <c r="M13" s="3" t="s">
         <v>17</v>
@@ -1895,49 +1973,49 @@
         <v>65</v>
       </c>
       <c r="S13" s="1" t="s">
-        <v>99</v>
-      </c>
-      <c r="T13" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="U13" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="T13" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="U13" s="3" t="s">
         <v>17</v>
       </c>
       <c r="V13" s="2">
-        <v>0</v>
+        <v>19500000</v>
       </c>
       <c r="W13" s="2">
-        <v>0</v>
+        <v>20240930</v>
       </c>
     </row>
     <row r="14" spans="1:23">
-      <c r="A14" s="34" t="s">
-        <v>68</v>
-      </c>
-      <c r="B14" s="4" t="s">
-        <v>29</v>
+      <c r="A14" s="18" t="s">
+        <v>30</v>
+      </c>
+      <c r="B14" s="37" t="s">
+        <v>25</v>
       </c>
       <c r="C14" s="24" t="s">
+        <v>104</v>
+      </c>
+      <c r="D14" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E14" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="F14" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="G14" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="H14" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="I14" s="24" t="s">
         <v>62</v>
       </c>
-      <c r="D14" s="3" t="s">
-        <v>63</v>
-      </c>
-      <c r="E14" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="F14" s="3" t="s">
-        <v>64</v>
-      </c>
-      <c r="G14" s="34" t="s">
-        <v>78</v>
-      </c>
-      <c r="H14" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="I14" s="24" t="s">
-        <v>66</v>
-      </c>
       <c r="J14" s="3" t="s">
         <v>63</v>
       </c>
@@ -1953,7 +2031,7 @@
       <c r="N14" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="O14" s="26" t="s">
+      <c r="O14" s="30" t="s">
         <v>53</v>
       </c>
       <c r="P14" s="30" t="s">
@@ -1968,10 +2046,10 @@
       <c r="S14" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="T14" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="U14" s="2" t="s">
+      <c r="T14" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="U14" s="3" t="s">
         <v>17</v>
       </c>
       <c r="V14" s="2">
@@ -1982,32 +2060,32 @@
       </c>
     </row>
     <row r="15" spans="1:23">
-      <c r="A15" s="34" t="s">
-        <v>69</v>
-      </c>
-      <c r="B15" s="4" t="s">
+      <c r="A15" s="18" t="s">
+        <v>40</v>
+      </c>
+      <c r="B15" s="37" t="s">
         <v>26</v>
       </c>
       <c r="C15" s="24" t="s">
+        <v>104</v>
+      </c>
+      <c r="D15" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E15" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="F15" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="G15" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="H15" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="I15" s="24" t="s">
         <v>62</v>
-      </c>
-      <c r="D15" s="3" t="s">
-        <v>63</v>
-      </c>
-      <c r="E15" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="F15" s="3" t="s">
-        <v>64</v>
-      </c>
-      <c r="G15" s="34" t="s">
-        <v>78</v>
-      </c>
-      <c r="H15" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="I15" s="24" t="s">
-        <v>66</v>
       </c>
       <c r="J15" s="3" t="s">
         <v>63</v>
@@ -2039,10 +2117,10 @@
       <c r="S15" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="T15" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="U15" s="2" t="s">
+      <c r="T15" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="U15" s="3" t="s">
         <v>17</v>
       </c>
       <c r="V15" s="2">
@@ -2053,32 +2131,32 @@
       </c>
     </row>
     <row r="16" spans="1:23">
-      <c r="A16" s="34" t="s">
-        <v>70</v>
-      </c>
-      <c r="B16" s="4" t="s">
+      <c r="A16" s="18" t="s">
+        <v>41</v>
+      </c>
+      <c r="B16" s="37" t="s">
         <v>27</v>
       </c>
       <c r="C16" s="24" t="s">
+        <v>104</v>
+      </c>
+      <c r="D16" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E16" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="F16" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="G16" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="H16" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="I16" s="24" t="s">
         <v>62</v>
-      </c>
-      <c r="D16" s="3" t="s">
-        <v>63</v>
-      </c>
-      <c r="E16" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="F16" s="3" t="s">
-        <v>64</v>
-      </c>
-      <c r="G16" s="34" t="s">
-        <v>78</v>
-      </c>
-      <c r="H16" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="I16" s="24" t="s">
-        <v>66</v>
       </c>
       <c r="J16" s="3" t="s">
         <v>63</v>
@@ -2110,10 +2188,10 @@
       <c r="S16" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="T16" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="U16" s="2" t="s">
+      <c r="T16" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="U16" s="3" t="s">
         <v>17</v>
       </c>
       <c r="V16" s="2">
@@ -2124,32 +2202,32 @@
       </c>
     </row>
     <row r="17" spans="1:23">
-      <c r="A17" s="34" t="s">
-        <v>71</v>
-      </c>
-      <c r="B17" s="4" t="s">
-        <v>51</v>
+      <c r="A17" s="18" t="s">
+        <v>42</v>
+      </c>
+      <c r="B17" s="37" t="s">
+        <v>28</v>
       </c>
       <c r="C17" s="24" t="s">
+        <v>104</v>
+      </c>
+      <c r="D17" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E17" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="F17" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="G17" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="H17" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="I17" s="24" t="s">
         <v>62</v>
-      </c>
-      <c r="D17" s="3" t="s">
-        <v>63</v>
-      </c>
-      <c r="E17" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="F17" s="3" t="s">
-        <v>64</v>
-      </c>
-      <c r="G17" s="34" t="s">
-        <v>78</v>
-      </c>
-      <c r="H17" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="I17" s="24" t="s">
-        <v>66</v>
       </c>
       <c r="J17" s="3" t="s">
         <v>63</v>
@@ -2181,10 +2259,10 @@
       <c r="S17" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="T17" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="U17" s="2" t="s">
+      <c r="T17" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="U17" s="3" t="s">
         <v>17</v>
       </c>
       <c r="V17" s="2">
@@ -2195,32 +2273,32 @@
       </c>
     </row>
     <row r="18" spans="1:23">
-      <c r="A18" s="34" t="s">
-        <v>72</v>
+      <c r="A18" s="18" t="s">
+        <v>43</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>52</v>
+        <v>29</v>
       </c>
       <c r="C18" s="24" t="s">
+        <v>104</v>
+      </c>
+      <c r="D18" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E18" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="F18" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="G18" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="H18" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="I18" s="24" t="s">
         <v>62</v>
-      </c>
-      <c r="D18" s="3" t="s">
-        <v>63</v>
-      </c>
-      <c r="E18" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="F18" s="3" t="s">
-        <v>64</v>
-      </c>
-      <c r="G18" s="34" t="s">
-        <v>78</v>
-      </c>
-      <c r="H18" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="I18" s="24" t="s">
-        <v>66</v>
       </c>
       <c r="J18" s="3" t="s">
         <v>63</v>
@@ -2252,10 +2330,10 @@
       <c r="S18" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="T18" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="U18" s="2" t="s">
+      <c r="T18" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="U18" s="3" t="s">
         <v>17</v>
       </c>
       <c r="V18" s="2">
@@ -2266,32 +2344,32 @@
       </c>
     </row>
     <row r="19" spans="1:23">
-      <c r="A19" s="34" t="s">
-        <v>73</v>
+      <c r="A19" s="18" t="s">
+        <v>44</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>28</v>
+        <v>51</v>
       </c>
       <c r="C19" s="24" t="s">
+        <v>104</v>
+      </c>
+      <c r="D19" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E19" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="F19" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="G19" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="H19" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="I19" s="24" t="s">
         <v>62</v>
-      </c>
-      <c r="D19" s="3" t="s">
-        <v>63</v>
-      </c>
-      <c r="E19" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="F19" s="3" t="s">
-        <v>64</v>
-      </c>
-      <c r="G19" s="34" t="s">
-        <v>78</v>
-      </c>
-      <c r="H19" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="I19" s="24" t="s">
-        <v>66</v>
       </c>
       <c r="J19" s="3" t="s">
         <v>63</v>
@@ -2323,10 +2401,10 @@
       <c r="S19" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="T19" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="U19" s="2" t="s">
+      <c r="T19" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="U19" s="3" t="s">
         <v>17</v>
       </c>
       <c r="V19" s="2">
@@ -2337,32 +2415,32 @@
       </c>
     </row>
     <row r="20" spans="1:23">
-      <c r="A20" s="34" t="s">
-        <v>74</v>
+      <c r="A20" s="18" t="s">
+        <v>49</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>23</v>
+        <v>52</v>
       </c>
       <c r="C20" s="24" t="s">
+        <v>104</v>
+      </c>
+      <c r="D20" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E20" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="F20" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="G20" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="H20" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="I20" s="24" t="s">
         <v>62</v>
-      </c>
-      <c r="D20" s="3" t="s">
-        <v>63</v>
-      </c>
-      <c r="E20" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="F20" s="3" t="s">
-        <v>64</v>
-      </c>
-      <c r="G20" s="34" t="s">
-        <v>78</v>
-      </c>
-      <c r="H20" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="I20" s="24" t="s">
-        <v>66</v>
       </c>
       <c r="J20" s="3" t="s">
         <v>63</v>
@@ -2394,10 +2472,10 @@
       <c r="S20" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="T20" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="U20" s="2" t="s">
+      <c r="T20" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="U20" s="3" t="s">
         <v>17</v>
       </c>
       <c r="V20" s="2">
@@ -2408,32 +2486,32 @@
       </c>
     </row>
     <row r="21" spans="1:23">
-      <c r="A21" s="34" t="s">
-        <v>75</v>
-      </c>
-      <c r="B21" s="4" t="s">
-        <v>55</v>
+      <c r="A21" s="32" t="s">
+        <v>54</v>
+      </c>
+      <c r="B21" s="37" t="s">
+        <v>23</v>
       </c>
       <c r="C21" s="24" t="s">
+        <v>104</v>
+      </c>
+      <c r="D21" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E21" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="F21" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="G21" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="H21" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="I21" s="24" t="s">
         <v>62</v>
-      </c>
-      <c r="D21" s="3" t="s">
-        <v>63</v>
-      </c>
-      <c r="E21" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="F21" s="3" t="s">
-        <v>64</v>
-      </c>
-      <c r="G21" s="34" t="s">
-        <v>78</v>
-      </c>
-      <c r="H21" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="I21" s="24" t="s">
-        <v>66</v>
       </c>
       <c r="J21" s="3" t="s">
         <v>63</v>
@@ -2465,10 +2543,10 @@
       <c r="S21" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="T21" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="U21" s="2" t="s">
+      <c r="T21" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="U21" s="3" t="s">
         <v>17</v>
       </c>
       <c r="V21" s="2">
@@ -2479,32 +2557,32 @@
       </c>
     </row>
     <row r="22" spans="1:23">
-      <c r="A22" s="34" t="s">
-        <v>76</v>
+      <c r="A22" s="32" t="s">
+        <v>58</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C22" s="24" t="s">
+        <v>104</v>
+      </c>
+      <c r="D22" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E22" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="F22" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="G22" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="H22" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="I22" s="24" t="s">
         <v>62</v>
-      </c>
-      <c r="D22" s="3" t="s">
-        <v>63</v>
-      </c>
-      <c r="E22" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="F22" s="3" t="s">
-        <v>64</v>
-      </c>
-      <c r="G22" s="34" t="s">
-        <v>78</v>
-      </c>
-      <c r="H22" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="I22" s="24" t="s">
-        <v>66</v>
       </c>
       <c r="J22" s="3" t="s">
         <v>63</v>
@@ -2536,10 +2614,10 @@
       <c r="S22" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="T22" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="U22" s="2" t="s">
+      <c r="T22" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="U22" s="3" t="s">
         <v>17</v>
       </c>
       <c r="V22" s="2">
@@ -2550,32 +2628,32 @@
       </c>
     </row>
     <row r="23" spans="1:23">
-      <c r="A23" s="34" t="s">
-        <v>77</v>
+      <c r="A23" s="32" t="s">
+        <v>59</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C23" s="24" t="s">
+        <v>104</v>
+      </c>
+      <c r="D23" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E23" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="F23" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="G23" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="H23" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="I23" s="24" t="s">
         <v>62</v>
-      </c>
-      <c r="D23" s="3" t="s">
-        <v>63</v>
-      </c>
-      <c r="E23" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="F23" s="3" t="s">
-        <v>64</v>
-      </c>
-      <c r="G23" s="34" t="s">
-        <v>78</v>
-      </c>
-      <c r="H23" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="I23" s="24" t="s">
-        <v>66</v>
       </c>
       <c r="J23" s="3" t="s">
         <v>63</v>
@@ -2607,51 +2685,51 @@
       <c r="S23" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="T23" s="2" t="s">
-        <v>83</v>
-      </c>
-      <c r="U23" s="2" t="s">
-        <v>83</v>
+      <c r="T23" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="U23" s="3" t="s">
+        <v>17</v>
       </c>
       <c r="V23" s="2">
-        <v>0</v>
+        <v>19500000</v>
       </c>
       <c r="W23" s="2">
-        <v>0</v>
+        <v>20240930</v>
       </c>
     </row>
     <row r="24" spans="1:23">
-      <c r="A24" s="34" t="s">
-        <v>79</v>
+      <c r="A24" s="32" t="s">
+        <v>60</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>25</v>
+        <v>57</v>
       </c>
       <c r="C24" s="24" t="s">
-        <v>61</v>
+        <v>104</v>
       </c>
       <c r="D24" s="3" t="s">
-        <v>63</v>
+        <v>0</v>
       </c>
       <c r="E24" s="3" t="s">
         <v>17</v>
       </c>
       <c r="F24" s="3" t="s">
-        <v>64</v>
-      </c>
-      <c r="G24" s="34" t="s">
-        <v>80</v>
+        <v>17</v>
+      </c>
+      <c r="G24" s="3" t="s">
+        <v>17</v>
       </c>
       <c r="H24" s="3" t="s">
-        <v>17</v>
+        <v>50</v>
       </c>
       <c r="I24" s="24" t="s">
-        <v>81</v>
+        <v>62</v>
       </c>
       <c r="J24" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="K24" s="34" t="s">
+      <c r="K24" s="3" t="s">
         <v>17</v>
       </c>
       <c r="L24" s="24" t="s">
@@ -2663,8 +2741,8 @@
       <c r="N24" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="O24" s="34" t="s">
-        <v>82</v>
+      <c r="O24" s="26" t="s">
+        <v>53</v>
       </c>
       <c r="P24" s="30" t="s">
         <v>53</v>
@@ -2678,11 +2756,11 @@
       <c r="S24" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="T24" s="2" t="s">
-        <v>83</v>
+      <c r="T24" s="3" t="s">
+        <v>86</v>
       </c>
       <c r="U24" s="2" t="s">
-        <v>83</v>
+        <v>100</v>
       </c>
       <c r="V24" s="2">
         <v>0</v>
@@ -2692,37 +2770,37 @@
       </c>
     </row>
     <row r="25" spans="1:23">
-      <c r="A25" s="34" t="s">
-        <v>88</v>
-      </c>
-      <c r="B25" s="4" t="s">
-        <v>29</v>
+      <c r="A25" s="38" t="s">
+        <v>67</v>
+      </c>
+      <c r="B25" s="17" t="s">
+        <v>101</v>
       </c>
       <c r="C25" s="24" t="s">
-        <v>61</v>
+        <v>104</v>
       </c>
       <c r="D25" s="3" t="s">
-        <v>63</v>
+        <v>0</v>
       </c>
       <c r="E25" s="3" t="s">
         <v>17</v>
       </c>
       <c r="F25" s="3" t="s">
-        <v>64</v>
-      </c>
-      <c r="G25" s="34" t="s">
-        <v>80</v>
+        <v>17</v>
+      </c>
+      <c r="G25" s="3" t="s">
+        <v>17</v>
       </c>
       <c r="H25" s="3" t="s">
-        <v>17</v>
+        <v>50</v>
       </c>
       <c r="I25" s="24" t="s">
-        <v>81</v>
+        <v>62</v>
       </c>
       <c r="J25" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="K25" s="34" t="s">
+      <c r="K25" s="3" t="s">
         <v>17</v>
       </c>
       <c r="L25" s="24" t="s">
@@ -2734,8 +2812,8 @@
       <c r="N25" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="O25" s="34" t="s">
-        <v>82</v>
+      <c r="O25" s="26" t="s">
+        <v>53</v>
       </c>
       <c r="P25" s="30" t="s">
         <v>53</v>
@@ -2749,28 +2827,28 @@
       <c r="S25" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="T25" s="2" t="s">
-        <v>83</v>
-      </c>
-      <c r="U25" s="2" t="s">
-        <v>83</v>
+      <c r="T25" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="U25" s="3" t="s">
+        <v>17</v>
       </c>
       <c r="V25" s="2">
-        <v>0</v>
+        <v>19500000</v>
       </c>
       <c r="W25" s="2">
-        <v>0</v>
+        <v>20240930</v>
       </c>
     </row>
     <row r="26" spans="1:23">
       <c r="A26" s="34" t="s">
-        <v>89</v>
+        <v>67</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C26" s="24" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="D26" s="3" t="s">
         <v>63</v>
@@ -2782,18 +2860,18 @@
         <v>64</v>
       </c>
       <c r="G26" s="34" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="H26" s="3" t="s">
         <v>17</v>
       </c>
       <c r="I26" s="24" t="s">
-        <v>81</v>
+        <v>66</v>
       </c>
       <c r="J26" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="K26" s="34" t="s">
+      <c r="K26" s="3" t="s">
         <v>17</v>
       </c>
       <c r="L26" s="24" t="s">
@@ -2805,8 +2883,8 @@
       <c r="N26" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="O26" s="34" t="s">
-        <v>82</v>
+      <c r="O26" s="26" t="s">
+        <v>53</v>
       </c>
       <c r="P26" s="30" t="s">
         <v>53</v>
@@ -2821,10 +2899,10 @@
         <v>99</v>
       </c>
       <c r="T26" s="2" t="s">
-        <v>83</v>
+        <v>17</v>
       </c>
       <c r="U26" s="2" t="s">
-        <v>83</v>
+        <v>17</v>
       </c>
       <c r="V26" s="2">
         <v>0</v>
@@ -2835,13 +2913,13 @@
     </row>
     <row r="27" spans="1:23">
       <c r="A27" s="34" t="s">
-        <v>90</v>
+        <v>68</v>
       </c>
       <c r="B27" s="4" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="C27" s="24" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="D27" s="3" t="s">
         <v>63</v>
@@ -2853,18 +2931,18 @@
         <v>64</v>
       </c>
       <c r="G27" s="34" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="H27" s="3" t="s">
         <v>17</v>
       </c>
       <c r="I27" s="24" t="s">
-        <v>81</v>
+        <v>66</v>
       </c>
       <c r="J27" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="K27" s="34" t="s">
+      <c r="K27" s="3" t="s">
         <v>17</v>
       </c>
       <c r="L27" s="24" t="s">
@@ -2876,8 +2954,8 @@
       <c r="N27" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="O27" s="34" t="s">
-        <v>82</v>
+      <c r="O27" s="26" t="s">
+        <v>53</v>
       </c>
       <c r="P27" s="30" t="s">
         <v>53</v>
@@ -2892,10 +2970,10 @@
         <v>99</v>
       </c>
       <c r="T27" s="2" t="s">
-        <v>83</v>
+        <v>17</v>
       </c>
       <c r="U27" s="2" t="s">
-        <v>83</v>
+        <v>17</v>
       </c>
       <c r="V27" s="2">
         <v>0</v>
@@ -2906,13 +2984,13 @@
     </row>
     <row r="28" spans="1:23">
       <c r="A28" s="34" t="s">
-        <v>91</v>
+        <v>69</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>51</v>
+        <v>26</v>
       </c>
       <c r="C28" s="24" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="D28" s="3" t="s">
         <v>63</v>
@@ -2924,18 +3002,18 @@
         <v>64</v>
       </c>
       <c r="G28" s="34" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="H28" s="3" t="s">
         <v>17</v>
       </c>
       <c r="I28" s="24" t="s">
-        <v>81</v>
+        <v>66</v>
       </c>
       <c r="J28" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="K28" s="34" t="s">
+      <c r="K28" s="3" t="s">
         <v>17</v>
       </c>
       <c r="L28" s="24" t="s">
@@ -2947,8 +3025,8 @@
       <c r="N28" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="O28" s="34" t="s">
-        <v>82</v>
+      <c r="O28" s="26" t="s">
+        <v>53</v>
       </c>
       <c r="P28" s="30" t="s">
         <v>53</v>
@@ -2963,10 +3041,10 @@
         <v>99</v>
       </c>
       <c r="T28" s="2" t="s">
-        <v>83</v>
+        <v>17</v>
       </c>
       <c r="U28" s="2" t="s">
-        <v>83</v>
+        <v>17</v>
       </c>
       <c r="V28" s="2">
         <v>0</v>
@@ -2977,13 +3055,13 @@
     </row>
     <row r="29" spans="1:23">
       <c r="A29" s="34" t="s">
-        <v>92</v>
+        <v>70</v>
       </c>
       <c r="B29" s="4" t="s">
-        <v>52</v>
+        <v>27</v>
       </c>
       <c r="C29" s="24" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="D29" s="3" t="s">
         <v>63</v>
@@ -2995,18 +3073,18 @@
         <v>64</v>
       </c>
       <c r="G29" s="34" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="H29" s="3" t="s">
         <v>17</v>
       </c>
       <c r="I29" s="24" t="s">
-        <v>81</v>
+        <v>66</v>
       </c>
       <c r="J29" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="K29" s="34" t="s">
+      <c r="K29" s="3" t="s">
         <v>17</v>
       </c>
       <c r="L29" s="24" t="s">
@@ -3018,8 +3096,8 @@
       <c r="N29" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="O29" s="34" t="s">
-        <v>82</v>
+      <c r="O29" s="26" t="s">
+        <v>53</v>
       </c>
       <c r="P29" s="30" t="s">
         <v>53</v>
@@ -3034,10 +3112,10 @@
         <v>99</v>
       </c>
       <c r="T29" s="2" t="s">
-        <v>83</v>
+        <v>17</v>
       </c>
       <c r="U29" s="2" t="s">
-        <v>83</v>
+        <v>17</v>
       </c>
       <c r="V29" s="2">
         <v>0</v>
@@ -3048,13 +3126,13 @@
     </row>
     <row r="30" spans="1:23">
       <c r="A30" s="34" t="s">
-        <v>93</v>
+        <v>71</v>
       </c>
       <c r="B30" s="4" t="s">
-        <v>28</v>
+        <v>51</v>
       </c>
       <c r="C30" s="24" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="D30" s="3" t="s">
         <v>63</v>
@@ -3066,18 +3144,18 @@
         <v>64</v>
       </c>
       <c r="G30" s="34" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="H30" s="3" t="s">
         <v>17</v>
       </c>
       <c r="I30" s="24" t="s">
-        <v>81</v>
+        <v>66</v>
       </c>
       <c r="J30" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="K30" s="34" t="s">
+      <c r="K30" s="3" t="s">
         <v>17</v>
       </c>
       <c r="L30" s="24" t="s">
@@ -3089,8 +3167,8 @@
       <c r="N30" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="O30" s="34" t="s">
-        <v>82</v>
+      <c r="O30" s="26" t="s">
+        <v>53</v>
       </c>
       <c r="P30" s="30" t="s">
         <v>53</v>
@@ -3105,10 +3183,10 @@
         <v>99</v>
       </c>
       <c r="T30" s="2" t="s">
-        <v>83</v>
+        <v>17</v>
       </c>
       <c r="U30" s="2" t="s">
-        <v>83</v>
+        <v>17</v>
       </c>
       <c r="V30" s="2">
         <v>0</v>
@@ -3119,13 +3197,13 @@
     </row>
     <row r="31" spans="1:23">
       <c r="A31" s="34" t="s">
-        <v>94</v>
+        <v>72</v>
       </c>
       <c r="B31" s="4" t="s">
-        <v>23</v>
+        <v>52</v>
       </c>
       <c r="C31" s="24" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="D31" s="3" t="s">
         <v>63</v>
@@ -3137,18 +3215,18 @@
         <v>64</v>
       </c>
       <c r="G31" s="34" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="H31" s="3" t="s">
         <v>17</v>
       </c>
       <c r="I31" s="24" t="s">
-        <v>81</v>
+        <v>66</v>
       </c>
       <c r="J31" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="K31" s="34" t="s">
+      <c r="K31" s="3" t="s">
         <v>17</v>
       </c>
       <c r="L31" s="24" t="s">
@@ -3160,8 +3238,8 @@
       <c r="N31" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="O31" s="34" t="s">
-        <v>82</v>
+      <c r="O31" s="26" t="s">
+        <v>53</v>
       </c>
       <c r="P31" s="30" t="s">
         <v>53</v>
@@ -3176,10 +3254,10 @@
         <v>99</v>
       </c>
       <c r="T31" s="2" t="s">
-        <v>83</v>
+        <v>17</v>
       </c>
       <c r="U31" s="2" t="s">
-        <v>83</v>
+        <v>17</v>
       </c>
       <c r="V31" s="2">
         <v>0</v>
@@ -3190,13 +3268,13 @@
     </row>
     <row r="32" spans="1:23">
       <c r="A32" s="34" t="s">
-        <v>95</v>
+        <v>73</v>
       </c>
       <c r="B32" s="4" t="s">
-        <v>55</v>
+        <v>28</v>
       </c>
       <c r="C32" s="24" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="D32" s="3" t="s">
         <v>63</v>
@@ -3208,18 +3286,18 @@
         <v>64</v>
       </c>
       <c r="G32" s="34" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="H32" s="3" t="s">
         <v>17</v>
       </c>
       <c r="I32" s="24" t="s">
-        <v>81</v>
+        <v>66</v>
       </c>
       <c r="J32" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="K32" s="34" t="s">
+      <c r="K32" s="3" t="s">
         <v>17</v>
       </c>
       <c r="L32" s="24" t="s">
@@ -3231,8 +3309,8 @@
       <c r="N32" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="O32" s="34" t="s">
-        <v>82</v>
+      <c r="O32" s="26" t="s">
+        <v>53</v>
       </c>
       <c r="P32" s="30" t="s">
         <v>53</v>
@@ -3247,10 +3325,10 @@
         <v>99</v>
       </c>
       <c r="T32" s="2" t="s">
-        <v>84</v>
+        <v>17</v>
       </c>
       <c r="U32" s="2" t="s">
-        <v>83</v>
+        <v>17</v>
       </c>
       <c r="V32" s="2">
         <v>0</v>
@@ -3261,13 +3339,13 @@
     </row>
     <row r="33" spans="1:23">
       <c r="A33" s="34" t="s">
-        <v>96</v>
+        <v>74</v>
       </c>
       <c r="B33" s="4" t="s">
-        <v>56</v>
+        <v>23</v>
       </c>
       <c r="C33" s="24" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="D33" s="3" t="s">
         <v>63</v>
@@ -3279,18 +3357,18 @@
         <v>64</v>
       </c>
       <c r="G33" s="34" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="H33" s="3" t="s">
         <v>17</v>
       </c>
       <c r="I33" s="24" t="s">
-        <v>81</v>
+        <v>66</v>
       </c>
       <c r="J33" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="K33" s="34" t="s">
+      <c r="K33" s="3" t="s">
         <v>17</v>
       </c>
       <c r="L33" s="24" t="s">
@@ -3302,8 +3380,8 @@
       <c r="N33" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="O33" s="34" t="s">
-        <v>82</v>
+      <c r="O33" s="26" t="s">
+        <v>53</v>
       </c>
       <c r="P33" s="30" t="s">
         <v>53</v>
@@ -3318,27 +3396,27 @@
         <v>99</v>
       </c>
       <c r="T33" s="2" t="s">
-        <v>53</v>
+        <v>17</v>
       </c>
       <c r="U33" s="2" t="s">
-        <v>83</v>
+        <v>17</v>
       </c>
       <c r="V33" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="W33" s="2">
-        <v>99999999</v>
+        <v>0</v>
       </c>
     </row>
     <row r="34" spans="1:23">
       <c r="A34" s="34" t="s">
-        <v>97</v>
+        <v>75</v>
       </c>
       <c r="B34" s="4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C34" s="24" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="D34" s="3" t="s">
         <v>63</v>
@@ -3350,18 +3428,18 @@
         <v>64</v>
       </c>
       <c r="G34" s="34" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="H34" s="3" t="s">
         <v>17</v>
       </c>
       <c r="I34" s="24" t="s">
-        <v>81</v>
+        <v>66</v>
       </c>
       <c r="J34" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="K34" s="34" t="s">
+      <c r="K34" s="3" t="s">
         <v>17</v>
       </c>
       <c r="L34" s="24" t="s">
@@ -3373,8 +3451,8 @@
       <c r="N34" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="O34" s="34" t="s">
-        <v>82</v>
+      <c r="O34" s="26" t="s">
+        <v>53</v>
       </c>
       <c r="P34" s="30" t="s">
         <v>53</v>
@@ -3388,28 +3466,28 @@
       <c r="S34" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="T34" s="35" t="s">
-        <v>85</v>
+      <c r="T34" s="2" t="s">
+        <v>17</v>
       </c>
       <c r="U34" s="2" t="s">
-        <v>83</v>
+        <v>17</v>
       </c>
       <c r="V34" s="2">
-        <v>19240101</v>
+        <v>0</v>
       </c>
       <c r="W34" s="2">
-        <v>20240101</v>
+        <v>0</v>
       </c>
     </row>
     <row r="35" spans="1:23">
       <c r="A35" s="34" t="s">
-        <v>98</v>
+        <v>76</v>
       </c>
       <c r="B35" s="4" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C35" s="24" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="D35" s="3" t="s">
         <v>63</v>
@@ -3421,18 +3499,18 @@
         <v>64</v>
       </c>
       <c r="G35" s="34" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="H35" s="3" t="s">
         <v>17</v>
       </c>
       <c r="I35" s="24" t="s">
-        <v>81</v>
+        <v>66</v>
       </c>
       <c r="J35" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="K35" s="34" t="s">
+      <c r="K35" s="3" t="s">
         <v>17</v>
       </c>
       <c r="L35" s="24" t="s">
@@ -3444,8 +3522,8 @@
       <c r="N35" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="O35" s="34" t="s">
-        <v>82</v>
+      <c r="O35" s="26" t="s">
+        <v>53</v>
       </c>
       <c r="P35" s="30" t="s">
         <v>53</v>
@@ -3460,62 +3538,1009 @@
         <v>99</v>
       </c>
       <c r="T35" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="U35" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="V35" s="2">
+        <v>0</v>
+      </c>
+      <c r="W35" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36" spans="1:23">
+      <c r="A36" s="34" t="s">
+        <v>77</v>
+      </c>
+      <c r="B36" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="C36" s="24" t="s">
+        <v>62</v>
+      </c>
+      <c r="D36" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="E36" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="F36" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="G36" s="34" t="s">
+        <v>78</v>
+      </c>
+      <c r="H36" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="I36" s="24" t="s">
+        <v>66</v>
+      </c>
+      <c r="J36" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="K36" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="L36" s="24" t="s">
+        <v>64</v>
+      </c>
+      <c r="M36" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="N36" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="O36" s="26" t="s">
+        <v>53</v>
+      </c>
+      <c r="P36" s="30" t="s">
+        <v>53</v>
+      </c>
+      <c r="Q36" s="31" t="s">
+        <v>53</v>
+      </c>
+      <c r="R36" s="33" t="s">
+        <v>65</v>
+      </c>
+      <c r="S36" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="T36" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="U36" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="V36" s="2">
+        <v>0</v>
+      </c>
+      <c r="W36" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37" spans="1:23">
+      <c r="A37" s="34" t="s">
+        <v>79</v>
+      </c>
+      <c r="B37" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="C37" s="24" t="s">
+        <v>61</v>
+      </c>
+      <c r="D37" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="E37" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="F37" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="G37" s="34" t="s">
+        <v>80</v>
+      </c>
+      <c r="H37" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="I37" s="24" t="s">
+        <v>81</v>
+      </c>
+      <c r="J37" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="K37" s="34" t="s">
+        <v>17</v>
+      </c>
+      <c r="L37" s="24" t="s">
+        <v>64</v>
+      </c>
+      <c r="M37" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="N37" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="O37" s="34" t="s">
+        <v>82</v>
+      </c>
+      <c r="P37" s="30" t="s">
+        <v>53</v>
+      </c>
+      <c r="Q37" s="31" t="s">
+        <v>53</v>
+      </c>
+      <c r="R37" s="33" t="s">
+        <v>65</v>
+      </c>
+      <c r="S37" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="T37" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="U37" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="V37" s="2">
+        <v>0</v>
+      </c>
+      <c r="W37" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38" spans="1:23">
+      <c r="A38" s="34" t="s">
+        <v>88</v>
+      </c>
+      <c r="B38" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="C38" s="24" t="s">
+        <v>61</v>
+      </c>
+      <c r="D38" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="E38" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="F38" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="G38" s="34" t="s">
+        <v>80</v>
+      </c>
+      <c r="H38" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="I38" s="24" t="s">
+        <v>81</v>
+      </c>
+      <c r="J38" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="K38" s="34" t="s">
+        <v>17</v>
+      </c>
+      <c r="L38" s="24" t="s">
+        <v>64</v>
+      </c>
+      <c r="M38" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="N38" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="O38" s="34" t="s">
+        <v>82</v>
+      </c>
+      <c r="P38" s="30" t="s">
+        <v>53</v>
+      </c>
+      <c r="Q38" s="31" t="s">
+        <v>53</v>
+      </c>
+      <c r="R38" s="33" t="s">
+        <v>65</v>
+      </c>
+      <c r="S38" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="T38" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="U38" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="V38" s="2">
+        <v>0</v>
+      </c>
+      <c r="W38" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39" spans="1:23">
+      <c r="A39" s="34" t="s">
+        <v>89</v>
+      </c>
+      <c r="B39" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="C39" s="24" t="s">
+        <v>61</v>
+      </c>
+      <c r="D39" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="E39" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="F39" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="G39" s="34" t="s">
+        <v>80</v>
+      </c>
+      <c r="H39" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="I39" s="24" t="s">
+        <v>81</v>
+      </c>
+      <c r="J39" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="K39" s="34" t="s">
+        <v>17</v>
+      </c>
+      <c r="L39" s="24" t="s">
+        <v>64</v>
+      </c>
+      <c r="M39" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="N39" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="O39" s="34" t="s">
+        <v>82</v>
+      </c>
+      <c r="P39" s="30" t="s">
+        <v>53</v>
+      </c>
+      <c r="Q39" s="31" t="s">
+        <v>53</v>
+      </c>
+      <c r="R39" s="33" t="s">
+        <v>65</v>
+      </c>
+      <c r="S39" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="T39" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="U39" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="V39" s="2">
+        <v>0</v>
+      </c>
+      <c r="W39" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40" spans="1:23">
+      <c r="A40" s="34" t="s">
+        <v>90</v>
+      </c>
+      <c r="B40" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="C40" s="24" t="s">
+        <v>61</v>
+      </c>
+      <c r="D40" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="E40" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="F40" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="G40" s="34" t="s">
+        <v>80</v>
+      </c>
+      <c r="H40" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="I40" s="24" t="s">
+        <v>81</v>
+      </c>
+      <c r="J40" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="K40" s="34" t="s">
+        <v>17</v>
+      </c>
+      <c r="L40" s="24" t="s">
+        <v>64</v>
+      </c>
+      <c r="M40" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="N40" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="O40" s="34" t="s">
+        <v>82</v>
+      </c>
+      <c r="P40" s="30" t="s">
+        <v>53</v>
+      </c>
+      <c r="Q40" s="31" t="s">
+        <v>53</v>
+      </c>
+      <c r="R40" s="33" t="s">
+        <v>65</v>
+      </c>
+      <c r="S40" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="T40" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="U40" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="V40" s="2">
+        <v>0</v>
+      </c>
+      <c r="W40" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41" spans="1:23">
+      <c r="A41" s="34" t="s">
+        <v>91</v>
+      </c>
+      <c r="B41" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="C41" s="24" t="s">
+        <v>61</v>
+      </c>
+      <c r="D41" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="E41" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="F41" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="G41" s="34" t="s">
+        <v>80</v>
+      </c>
+      <c r="H41" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="I41" s="24" t="s">
+        <v>81</v>
+      </c>
+      <c r="J41" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="K41" s="34" t="s">
+        <v>17</v>
+      </c>
+      <c r="L41" s="24" t="s">
+        <v>64</v>
+      </c>
+      <c r="M41" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="N41" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="O41" s="34" t="s">
+        <v>82</v>
+      </c>
+      <c r="P41" s="30" t="s">
+        <v>53</v>
+      </c>
+      <c r="Q41" s="31" t="s">
+        <v>53</v>
+      </c>
+      <c r="R41" s="33" t="s">
+        <v>65</v>
+      </c>
+      <c r="S41" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="T41" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="U41" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="V41" s="2">
+        <v>0</v>
+      </c>
+      <c r="W41" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42" spans="1:23">
+      <c r="A42" s="34" t="s">
+        <v>92</v>
+      </c>
+      <c r="B42" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="C42" s="24" t="s">
+        <v>61</v>
+      </c>
+      <c r="D42" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="E42" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="F42" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="G42" s="34" t="s">
+        <v>80</v>
+      </c>
+      <c r="H42" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="I42" s="24" t="s">
+        <v>81</v>
+      </c>
+      <c r="J42" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="K42" s="34" t="s">
+        <v>17</v>
+      </c>
+      <c r="L42" s="24" t="s">
+        <v>64</v>
+      </c>
+      <c r="M42" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="N42" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="O42" s="34" t="s">
+        <v>82</v>
+      </c>
+      <c r="P42" s="30" t="s">
+        <v>53</v>
+      </c>
+      <c r="Q42" s="31" t="s">
+        <v>53</v>
+      </c>
+      <c r="R42" s="33" t="s">
+        <v>65</v>
+      </c>
+      <c r="S42" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="T42" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="U42" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="V42" s="2">
+        <v>0</v>
+      </c>
+      <c r="W42" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43" spans="1:23">
+      <c r="A43" s="34" t="s">
+        <v>93</v>
+      </c>
+      <c r="B43" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="C43" s="24" t="s">
+        <v>61</v>
+      </c>
+      <c r="D43" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="E43" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="F43" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="G43" s="34" t="s">
+        <v>80</v>
+      </c>
+      <c r="H43" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="I43" s="24" t="s">
+        <v>81</v>
+      </c>
+      <c r="J43" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="K43" s="34" t="s">
+        <v>17</v>
+      </c>
+      <c r="L43" s="24" t="s">
+        <v>64</v>
+      </c>
+      <c r="M43" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="N43" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="O43" s="34" t="s">
+        <v>82</v>
+      </c>
+      <c r="P43" s="30" t="s">
+        <v>53</v>
+      </c>
+      <c r="Q43" s="31" t="s">
+        <v>53</v>
+      </c>
+      <c r="R43" s="33" t="s">
+        <v>65</v>
+      </c>
+      <c r="S43" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="T43" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="U43" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="V43" s="2">
+        <v>0</v>
+      </c>
+      <c r="W43" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44" spans="1:23">
+      <c r="A44" s="34" t="s">
+        <v>94</v>
+      </c>
+      <c r="B44" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="C44" s="24" t="s">
+        <v>61</v>
+      </c>
+      <c r="D44" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="E44" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="F44" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="G44" s="34" t="s">
+        <v>80</v>
+      </c>
+      <c r="H44" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="I44" s="24" t="s">
+        <v>81</v>
+      </c>
+      <c r="J44" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="K44" s="34" t="s">
+        <v>17</v>
+      </c>
+      <c r="L44" s="24" t="s">
+        <v>64</v>
+      </c>
+      <c r="M44" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="N44" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="O44" s="34" t="s">
+        <v>82</v>
+      </c>
+      <c r="P44" s="30" t="s">
+        <v>53</v>
+      </c>
+      <c r="Q44" s="31" t="s">
+        <v>53</v>
+      </c>
+      <c r="R44" s="33" t="s">
+        <v>65</v>
+      </c>
+      <c r="S44" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="T44" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="U44" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="V44" s="2">
+        <v>0</v>
+      </c>
+      <c r="W44" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45" spans="1:23">
+      <c r="A45" s="34" t="s">
+        <v>95</v>
+      </c>
+      <c r="B45" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="C45" s="24" t="s">
+        <v>61</v>
+      </c>
+      <c r="D45" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="E45" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="F45" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="G45" s="34" t="s">
+        <v>80</v>
+      </c>
+      <c r="H45" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="I45" s="24" t="s">
+        <v>81</v>
+      </c>
+      <c r="J45" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="K45" s="34" t="s">
+        <v>17</v>
+      </c>
+      <c r="L45" s="24" t="s">
+        <v>64</v>
+      </c>
+      <c r="M45" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="N45" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="O45" s="34" t="s">
+        <v>82</v>
+      </c>
+      <c r="P45" s="30" t="s">
+        <v>53</v>
+      </c>
+      <c r="Q45" s="31" t="s">
+        <v>53</v>
+      </c>
+      <c r="R45" s="33" t="s">
+        <v>65</v>
+      </c>
+      <c r="S45" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="T45" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="U45" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="V45" s="2">
+        <v>0</v>
+      </c>
+      <c r="W45" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46" spans="1:23">
+      <c r="A46" s="34" t="s">
+        <v>96</v>
+      </c>
+      <c r="B46" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="C46" s="24" t="s">
+        <v>61</v>
+      </c>
+      <c r="D46" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="E46" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="F46" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="G46" s="34" t="s">
+        <v>80</v>
+      </c>
+      <c r="H46" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="I46" s="24" t="s">
+        <v>81</v>
+      </c>
+      <c r="J46" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="K46" s="34" t="s">
+        <v>17</v>
+      </c>
+      <c r="L46" s="24" t="s">
+        <v>64</v>
+      </c>
+      <c r="M46" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="N46" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="O46" s="34" t="s">
+        <v>82</v>
+      </c>
+      <c r="P46" s="30" t="s">
+        <v>53</v>
+      </c>
+      <c r="Q46" s="31" t="s">
+        <v>53</v>
+      </c>
+      <c r="R46" s="33" t="s">
+        <v>65</v>
+      </c>
+      <c r="S46" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="T46" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="U46" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="V46" s="2">
+        <v>1</v>
+      </c>
+      <c r="W46" s="2">
+        <v>99999999</v>
+      </c>
+    </row>
+    <row r="47" spans="1:23">
+      <c r="A47" s="34" t="s">
+        <v>97</v>
+      </c>
+      <c r="B47" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="C47" s="24" t="s">
+        <v>61</v>
+      </c>
+      <c r="D47" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="E47" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="F47" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="G47" s="34" t="s">
+        <v>80</v>
+      </c>
+      <c r="H47" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="I47" s="24" t="s">
+        <v>81</v>
+      </c>
+      <c r="J47" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="K47" s="34" t="s">
+        <v>17</v>
+      </c>
+      <c r="L47" s="24" t="s">
+        <v>64</v>
+      </c>
+      <c r="M47" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="N47" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="O47" s="34" t="s">
+        <v>82</v>
+      </c>
+      <c r="P47" s="30" t="s">
+        <v>53</v>
+      </c>
+      <c r="Q47" s="31" t="s">
+        <v>53</v>
+      </c>
+      <c r="R47" s="33" t="s">
+        <v>65</v>
+      </c>
+      <c r="S47" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="T47" s="35" t="s">
+        <v>85</v>
+      </c>
+      <c r="U47" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="V47" s="2">
+        <v>19240101</v>
+      </c>
+      <c r="W47" s="2">
+        <v>20240101</v>
+      </c>
+    </row>
+    <row r="48" spans="1:23">
+      <c r="A48" s="34" t="s">
+        <v>98</v>
+      </c>
+      <c r="B48" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="C48" s="24" t="s">
+        <v>61</v>
+      </c>
+      <c r="D48" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="E48" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="F48" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="G48" s="34" t="s">
+        <v>80</v>
+      </c>
+      <c r="H48" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="I48" s="24" t="s">
+        <v>81</v>
+      </c>
+      <c r="J48" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="K48" s="34" t="s">
+        <v>17</v>
+      </c>
+      <c r="L48" s="24" t="s">
+        <v>64</v>
+      </c>
+      <c r="M48" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="N48" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="O48" s="34" t="s">
+        <v>82</v>
+      </c>
+      <c r="P48" s="30" t="s">
+        <v>53</v>
+      </c>
+      <c r="Q48" s="31" t="s">
+        <v>53</v>
+      </c>
+      <c r="R48" s="33" t="s">
+        <v>65</v>
+      </c>
+      <c r="S48" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="T48" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="U35" s="2" t="s">
+      <c r="U48" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="V35" s="2">
-        <v>0</v>
-      </c>
-      <c r="W35" s="2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="36" spans="1:23">
-      <c r="A36" s="16"/>
-      <c r="B36" s="4"/>
-      <c r="C36" s="3"/>
-      <c r="D36" s="3"/>
-      <c r="E36" s="3"/>
-      <c r="F36" s="3"/>
-      <c r="G36" s="11"/>
-      <c r="H36" s="15"/>
-      <c r="I36" s="13"/>
-      <c r="J36" s="3"/>
-      <c r="K36" s="3"/>
-      <c r="L36" s="14"/>
-      <c r="M36" s="12"/>
-      <c r="N36" s="3"/>
-      <c r="O36" s="6"/>
-      <c r="P36" s="7"/>
-      <c r="Q36" s="9"/>
-      <c r="R36" s="10"/>
-      <c r="S36" s="1"/>
-    </row>
-    <row r="37" spans="1:23">
-      <c r="A37" s="16"/>
-      <c r="B37" s="4"/>
-      <c r="C37" s="3"/>
-      <c r="D37" s="3"/>
-      <c r="E37" s="3"/>
-      <c r="F37" s="3"/>
-      <c r="G37" s="11"/>
-      <c r="H37" s="15"/>
-      <c r="I37" s="13"/>
-      <c r="J37" s="3"/>
-      <c r="K37" s="3"/>
-      <c r="L37" s="14"/>
-      <c r="M37" s="12"/>
-      <c r="N37" s="3"/>
-      <c r="O37" s="6"/>
-      <c r="P37" s="7"/>
-      <c r="Q37" s="9"/>
-      <c r="R37" s="10"/>
-      <c r="S37" s="1"/>
+      <c r="V48" s="2">
+        <v>0</v>
+      </c>
+      <c r="W48" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49" spans="1:19">
+      <c r="A49" s="39" t="s">
+        <v>102</v>
+      </c>
+      <c r="B49" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="C49" s="3"/>
+      <c r="D49" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="E49" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="F49" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="G49" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="H49" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="I49" s="13"/>
+      <c r="J49" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="K49" s="34" t="s">
+        <v>17</v>
+      </c>
+      <c r="L49" s="24" t="s">
+        <v>64</v>
+      </c>
+      <c r="M49" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="N49" s="3"/>
+      <c r="O49" s="6"/>
+      <c r="P49" s="7"/>
+      <c r="Q49" s="9"/>
+      <c r="R49" s="10"/>
+      <c r="S49" s="1" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="50" spans="1:19">
+      <c r="A50" s="16"/>
+      <c r="B50" s="4"/>
+      <c r="C50" s="3"/>
+      <c r="D50" s="3"/>
+      <c r="E50" s="3"/>
+      <c r="F50" s="3"/>
+      <c r="G50" s="11"/>
+      <c r="H50" s="15"/>
+      <c r="I50" s="13"/>
+      <c r="J50" s="3"/>
+      <c r="K50" s="3"/>
+      <c r="L50" s="14"/>
+      <c r="M50" s="12"/>
+      <c r="N50" s="3"/>
+      <c r="O50" s="6"/>
+      <c r="P50" s="7"/>
+      <c r="Q50" s="9"/>
+      <c r="R50" s="10"/>
+      <c r="S50" s="1"/>
     </row>
   </sheetData>
-  <phoneticPr fontId="26" type="noConversion"/>
+  <phoneticPr fontId="29" type="noConversion"/>
   <dataValidations count="4">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J1:J1048576" xr:uid="{39CDAD1A-527D-8A43-BFCC-4279C43AB355}">
       <formula1>"csv,json,parquet,avro,table,snowflake,redshift,adls,s3"</formula1>
@@ -3523,10 +4548,10 @@
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D1:D1048576" xr:uid="{0251E4F9-1266-42BB-802C-E032AD2F255C}">
       <formula1>"csv,json,parquet,avro,table,redshift,snowflake,adls,s3"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="S2:S37" xr:uid="{53648117-6315-BD4B-95C3-AF9A5887C458}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="S2:S50" xr:uid="{53648117-6315-BD4B-95C3-AF9A5887C458}">
       <formula1>"Y,N"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B1:B1048576" xr:uid="{A736D6D3-E056-442B-8A93-B37F82E798F4}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B26:B1048576 B1:B12 B14:B24" xr:uid="{A736D6D3-E056-442B-8A93-B37F82E798F4}">
       <formula1>"count_check,duplicate,null_value_check,uniqueness_check,records_present_only_in_source,records_present_only_target,data_compare,schema_check,name_check,column_range_check,column_value_reference_check"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>